<commit_message>
Add a description column to the client sheet
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Manussa-your-pieces.xlsx
+++ b/docs/Manussa-your-pieces.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -508,8 +508,9 @@
     <col width="6" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
     <col width="6" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="54" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -591,8 +592,13 @@
           <t>How should it be cleaned?</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>Describe it — what makes it special?</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="54" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Painted Capelet</t>
@@ -607,8 +613,9 @@
       <c r="H6" s="9" t="n"/>
       <c r="I6" s="10" t="n"/>
       <c r="J6" s="10" t="n"/>
-    </row>
-    <row r="7" ht="30" customHeight="1">
+      <c r="K6" s="10" t="n"/>
+    </row>
+    <row r="7" ht="54" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Column Gown</t>
@@ -623,8 +630,9 @@
       <c r="H7" s="9" t="n"/>
       <c r="I7" s="10" t="n"/>
       <c r="J7" s="10" t="n"/>
-    </row>
-    <row r="8" ht="30" customHeight="1">
+      <c r="K7" s="10" t="n"/>
+    </row>
+    <row r="8" ht="54" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Painted Corset Bodice</t>
@@ -639,8 +647,9 @@
       <c r="H8" s="9" t="n"/>
       <c r="I8" s="10" t="n"/>
       <c r="J8" s="10" t="n"/>
-    </row>
-    <row r="9" ht="30" customHeight="1">
+      <c r="K8" s="10" t="n"/>
+    </row>
+    <row r="9" ht="54" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Raw Silk Fluted Skirt</t>
@@ -655,8 +664,9 @@
       <c r="H9" s="9" t="n"/>
       <c r="I9" s="10" t="n"/>
       <c r="J9" s="10" t="n"/>
-    </row>
-    <row r="10" ht="30" customHeight="1">
+      <c r="K9" s="10" t="n"/>
+    </row>
+    <row r="10" ht="54" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Elegant Powerful Jacket</t>
@@ -671,8 +681,9 @@
       <c r="H10" s="9" t="n"/>
       <c r="I10" s="10" t="n"/>
       <c r="J10" s="10" t="n"/>
-    </row>
-    <row r="11" ht="30" customHeight="1">
+      <c r="K10" s="10" t="n"/>
+    </row>
+    <row r="11" ht="54" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Crimson Drive Jacket</t>
@@ -687,8 +698,9 @@
       <c r="H11" s="9" t="n"/>
       <c r="I11" s="10" t="n"/>
       <c r="J11" s="10" t="n"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
+      <c r="K11" s="10" t="n"/>
+    </row>
+    <row r="12" ht="54" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Men's Panelled Jacket</t>
@@ -703,8 +715,9 @@
       <c r="H12" s="9" t="n"/>
       <c r="I12" s="10" t="n"/>
       <c r="J12" s="10" t="n"/>
-    </row>
-    <row r="13" ht="30" customHeight="1">
+      <c r="K12" s="10" t="n"/>
+    </row>
+    <row r="13" ht="54" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Melting Paint Denim Jacket</t>
@@ -719,8 +732,9 @@
       <c r="H13" s="9" t="n"/>
       <c r="I13" s="10" t="n"/>
       <c r="J13" s="10" t="n"/>
-    </row>
-    <row r="14" ht="30" customHeight="1">
+      <c r="K13" s="10" t="n"/>
+    </row>
+    <row r="14" ht="54" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Indigo Panel Denim Jacket</t>
@@ -735,8 +749,9 @@
       <c r="H14" s="9" t="n"/>
       <c r="I14" s="10" t="n"/>
       <c r="J14" s="10" t="n"/>
-    </row>
-    <row r="15" ht="30" customHeight="1">
+      <c r="K14" s="10" t="n"/>
+    </row>
+    <row r="15" ht="54" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>New Traditional Patchwork Jacket</t>
@@ -751,8 +766,9 @@
       <c r="H15" s="9" t="n"/>
       <c r="I15" s="10" t="n"/>
       <c r="J15" s="10" t="n"/>
-    </row>
-    <row r="16" ht="30" customHeight="1">
+      <c r="K15" s="10" t="n"/>
+    </row>
+    <row r="16" ht="54" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Mosaic Peplum Top</t>
@@ -767,8 +783,9 @@
       <c r="H16" s="9" t="n"/>
       <c r="I16" s="10" t="n"/>
       <c r="J16" s="10" t="n"/>
-    </row>
-    <row r="17" ht="30" customHeight="1">
+      <c r="K16" s="10" t="n"/>
+    </row>
+    <row r="17" ht="54" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Coral Embroidered Gown</t>
@@ -783,8 +800,9 @@
       <c r="H17" s="9" t="n"/>
       <c r="I17" s="10" t="n"/>
       <c r="J17" s="10" t="n"/>
-    </row>
-    <row r="18" ht="30" customHeight="1">
+      <c r="K17" s="10" t="n"/>
+    </row>
+    <row r="18" ht="54" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
         <is>
           <t>Structured Peplum Vest</t>
@@ -799,6 +817,7 @@
       <c r="H18" s="9" t="n"/>
       <c r="I18" s="10" t="n"/>
       <c r="J18" s="10" t="n"/>
+      <c r="K18" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>